<commit_message>
feat - Used fuzzy matching for everything as opposed to mixing it with querying the pandas table. Created a separate extras table.
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -3103,7 +3103,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>DNS</t>
+          <t>52.86</t>
         </is>
       </c>
       <c r="G69" s="1" t="n">
@@ -6319,7 +6319,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>DNS</t>
+          <t>2.20.81</t>
         </is>
       </c>
       <c r="G151" s="1" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>1.27.75</t>
+          <t>1.32.88</t>
         </is>
       </c>
       <c r="G166" s="1" t="n">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>DNS</t>
+          <t>45.39</t>
         </is>
       </c>
       <c r="G261" s="1" t="n">
@@ -13921,7 +13921,7 @@
       </c>
       <c r="F345" s="2" t="inlineStr">
         <is>
-          <t>DNS</t>
+          <t>2.03.06</t>
         </is>
       </c>
       <c r="G345" s="1" t="n">
@@ -14475,7 +14475,7 @@
       </c>
       <c r="F359" s="2" t="inlineStr">
         <is>
-          <t>1.20.28</t>
+          <t>1.19.47</t>
         </is>
       </c>
       <c r="G359" s="1" t="n">
@@ -18227,7 +18227,7 @@
       </c>
       <c r="F455" s="2" t="inlineStr">
         <is>
-          <t>DNS</t>
+          <t>1.04.76</t>
         </is>
       </c>
       <c r="G455" s="1" t="n">
@@ -21170,7 +21170,7 @@
       </c>
       <c r="F530" s="2" t="inlineStr">
         <is>
-          <t>DNS</t>
+          <t>2.14.33</t>
         </is>
       </c>
       <c r="G530" s="1" t="n">
@@ -22040,7 +22040,7 @@
       </c>
       <c r="F552" s="2" t="inlineStr">
         <is>
-          <t>1.42.09</t>
+          <t>1.43.69</t>
         </is>
       </c>
       <c r="G552" s="1" t="n">
@@ -25829,7 +25829,7 @@
       </c>
       <c r="F649" s="2" t="inlineStr">
         <is>
-          <t>DNS</t>
+          <t>1.09.57</t>
         </is>
       </c>
       <c r="G649" s="1" t="n">
@@ -29047,7 +29047,7 @@
       </c>
       <c r="F731" s="2" t="inlineStr">
         <is>
-          <t>DNS</t>
+          <t>2.48.81</t>
         </is>
       </c>
       <c r="G731" s="1" t="n">
@@ -29876,7 +29876,7 @@
       </c>
       <c r="F752" s="2" t="inlineStr">
         <is>
-          <t>1.37.72</t>
+          <t>1.46.13</t>
         </is>
       </c>
       <c r="G752" s="1" t="n">
@@ -33394,7 +33394,7 @@
       </c>
       <c r="F842" s="2" t="inlineStr">
         <is>
-          <t>2.18.50</t>
+          <t>2.09.88</t>
         </is>
       </c>
       <c r="G842" s="1" t="n">
@@ -36296,7 +36296,7 @@
       </c>
       <c r="F916" s="2" t="inlineStr">
         <is>
-          <t>2.09.88</t>
+          <t>2.18.50</t>
         </is>
       </c>
       <c r="G916" s="1" t="n">
@@ -37084,7 +37084,7 @@
       </c>
       <c r="F936" s="2" t="inlineStr">
         <is>
-          <t>1.32.53</t>
+          <t>1.32.75</t>
         </is>
       </c>
       <c r="G936" s="1" t="n">

</xml_diff>

<commit_message>
refactor - Kept Leah's Tables separated when adding extra rows and only combine on output.
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -1891,7 +1891,9 @@
       <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="1" t="inlineStr"/>
       <c r="H38" s="1" t="inlineStr"/>
-      <c r="I38" s="1" t="inlineStr"/>
+      <c r="I38" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
@@ -1924,7 +1926,9 @@
       </c>
       <c r="G39" s="1" t="inlineStr"/>
       <c r="H39" s="1" t="inlineStr"/>
-      <c r="I39" s="1" t="inlineStr"/>
+      <c r="I39" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
@@ -1957,7 +1961,9 @@
       </c>
       <c r="G40" s="1" t="inlineStr"/>
       <c r="H40" s="1" t="inlineStr"/>
-      <c r="I40" s="1" t="inlineStr"/>
+      <c r="I40" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
@@ -1990,7 +1996,9 @@
       </c>
       <c r="G41" s="1" t="inlineStr"/>
       <c r="H41" s="1" t="inlineStr"/>
-      <c r="I41" s="1" t="inlineStr"/>
+      <c r="I41" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
@@ -2023,7 +2031,9 @@
       </c>
       <c r="G42" s="1" t="inlineStr"/>
       <c r="H42" s="1" t="inlineStr"/>
-      <c r="I42" s="1" t="inlineStr"/>
+      <c r="I42" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
@@ -2056,7 +2066,9 @@
       </c>
       <c r="G43" s="1" t="inlineStr"/>
       <c r="H43" s="1" t="inlineStr"/>
-      <c r="I43" s="1" t="inlineStr"/>
+      <c r="I43" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
@@ -3093,7 +3105,9 @@
       <c r="F70" s="2" t="inlineStr"/>
       <c r="G70" s="1" t="inlineStr"/>
       <c r="H70" s="1" t="inlineStr"/>
-      <c r="I70" s="1" t="inlineStr"/>
+      <c r="I70" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
@@ -3124,7 +3138,9 @@
       </c>
       <c r="G71" s="1" t="inlineStr"/>
       <c r="H71" s="1" t="inlineStr"/>
-      <c r="I71" s="1" t="inlineStr"/>
+      <c r="I71" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
@@ -4436,7 +4452,9 @@
       <c r="F105" s="2" t="inlineStr"/>
       <c r="G105" s="1" t="inlineStr"/>
       <c r="H105" s="1" t="inlineStr"/>
-      <c r="I105" s="1" t="inlineStr"/>
+      <c r="I105" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
@@ -4469,7 +4487,9 @@
       </c>
       <c r="G106" s="1" t="inlineStr"/>
       <c r="H106" s="1" t="inlineStr"/>
-      <c r="I106" s="1" t="inlineStr"/>
+      <c r="I106" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
@@ -4502,7 +4522,9 @@
       </c>
       <c r="G107" s="1" t="inlineStr"/>
       <c r="H107" s="1" t="inlineStr"/>
-      <c r="I107" s="1" t="inlineStr"/>
+      <c r="I107" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
@@ -5496,7 +5518,9 @@
       <c r="F133" s="2" t="inlineStr"/>
       <c r="G133" s="1" t="inlineStr"/>
       <c r="H133" s="1" t="inlineStr"/>
-      <c r="I133" s="1" t="inlineStr"/>
+      <c r="I133" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
@@ -5529,7 +5553,9 @@
       </c>
       <c r="G134" s="1" t="inlineStr"/>
       <c r="H134" s="1" t="inlineStr"/>
-      <c r="I134" s="1" t="inlineStr"/>
+      <c r="I134" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
@@ -5560,7 +5586,9 @@
       </c>
       <c r="G135" s="1" t="inlineStr"/>
       <c r="H135" s="1" t="inlineStr"/>
-      <c r="I135" s="1" t="inlineStr"/>
+      <c r="I135" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
@@ -5591,7 +5619,9 @@
       </c>
       <c r="G136" s="1" t="inlineStr"/>
       <c r="H136" s="1" t="inlineStr"/>
-      <c r="I136" s="1" t="inlineStr"/>
+      <c r="I136" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
@@ -5622,7 +5652,9 @@
       </c>
       <c r="G137" s="1" t="inlineStr"/>
       <c r="H137" s="1" t="inlineStr"/>
-      <c r="I137" s="1" t="inlineStr"/>
+      <c r="I137" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
@@ -6343,7 +6375,9 @@
       <c r="F156" s="2" t="inlineStr"/>
       <c r="G156" s="1" t="inlineStr"/>
       <c r="H156" s="1" t="inlineStr"/>
-      <c r="I156" s="1" t="inlineStr"/>
+      <c r="I156" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
@@ -6376,7 +6410,9 @@
       </c>
       <c r="G157" s="1" t="inlineStr"/>
       <c r="H157" s="1" t="inlineStr"/>
-      <c r="I157" s="1" t="inlineStr"/>
+      <c r="I157" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
@@ -6407,7 +6443,9 @@
       </c>
       <c r="G158" s="1" t="inlineStr"/>
       <c r="H158" s="1" t="inlineStr"/>
-      <c r="I158" s="1" t="inlineStr"/>
+      <c r="I158" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
@@ -6438,7 +6476,9 @@
       </c>
       <c r="G159" s="1" t="inlineStr"/>
       <c r="H159" s="1" t="inlineStr"/>
-      <c r="I159" s="1" t="inlineStr"/>
+      <c r="I159" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
@@ -6471,7 +6511,9 @@
       </c>
       <c r="G160" s="1" t="inlineStr"/>
       <c r="H160" s="1" t="inlineStr"/>
-      <c r="I160" s="1" t="inlineStr"/>
+      <c r="I160" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
@@ -6504,7 +6546,9 @@
       </c>
       <c r="G161" s="1" t="inlineStr"/>
       <c r="H161" s="1" t="inlineStr"/>
-      <c r="I161" s="1" t="inlineStr"/>
+      <c r="I161" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
@@ -7266,7 +7310,9 @@
       <c r="F181" s="2" t="inlineStr"/>
       <c r="G181" s="1" t="inlineStr"/>
       <c r="H181" s="1" t="inlineStr"/>
-      <c r="I181" s="1" t="inlineStr"/>
+      <c r="I181" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
@@ -7297,7 +7343,9 @@
       </c>
       <c r="G182" s="1" t="inlineStr"/>
       <c r="H182" s="1" t="inlineStr"/>
-      <c r="I182" s="1" t="inlineStr"/>
+      <c r="I182" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
@@ -7330,7 +7378,9 @@
       </c>
       <c r="G183" s="1" t="inlineStr"/>
       <c r="H183" s="1" t="inlineStr"/>
-      <c r="I183" s="1" t="inlineStr"/>
+      <c r="I183" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
@@ -7969,7 +8019,9 @@
       <c r="F200" s="2" t="inlineStr"/>
       <c r="G200" s="1" t="inlineStr"/>
       <c r="H200" s="1" t="inlineStr"/>
-      <c r="I200" s="1" t="inlineStr"/>
+      <c r="I200" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
@@ -8000,7 +8052,9 @@
       </c>
       <c r="G201" s="1" t="inlineStr"/>
       <c r="H201" s="1" t="inlineStr"/>
-      <c r="I201" s="1" t="inlineStr"/>
+      <c r="I201" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
@@ -8033,7 +8087,9 @@
       </c>
       <c r="G202" s="1" t="inlineStr"/>
       <c r="H202" s="1" t="inlineStr"/>
-      <c r="I202" s="1" t="inlineStr"/>
+      <c r="I202" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
@@ -8066,7 +8122,9 @@
       </c>
       <c r="G203" s="1" t="inlineStr"/>
       <c r="H203" s="1" t="inlineStr"/>
-      <c r="I203" s="1" t="inlineStr"/>
+      <c r="I203" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
@@ -8099,7 +8157,9 @@
       </c>
       <c r="G204" s="1" t="inlineStr"/>
       <c r="H204" s="1" t="inlineStr"/>
-      <c r="I204" s="1" t="inlineStr"/>
+      <c r="I204" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
@@ -8902,7 +8962,9 @@
       <c r="F225" s="2" t="inlineStr"/>
       <c r="G225" s="1" t="inlineStr"/>
       <c r="H225" s="1" t="inlineStr"/>
-      <c r="I225" s="1" t="inlineStr"/>
+      <c r="I225" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
@@ -8935,7 +8997,9 @@
       </c>
       <c r="G226" s="1" t="inlineStr"/>
       <c r="H226" s="1" t="inlineStr"/>
-      <c r="I226" s="1" t="inlineStr"/>
+      <c r="I226" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
@@ -8968,7 +9032,9 @@
       </c>
       <c r="G227" s="1" t="inlineStr"/>
       <c r="H227" s="1" t="inlineStr"/>
-      <c r="I227" s="1" t="inlineStr"/>
+      <c r="I227" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
@@ -9001,7 +9067,9 @@
       </c>
       <c r="G228" s="1" t="inlineStr"/>
       <c r="H228" s="1" t="inlineStr"/>
-      <c r="I228" s="1" t="inlineStr"/>
+      <c r="I228" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
@@ -10455,7 +10523,9 @@
       <c r="F266" s="2" t="inlineStr"/>
       <c r="G266" s="1" t="inlineStr"/>
       <c r="H266" s="1" t="inlineStr"/>
-      <c r="I266" s="1" t="inlineStr"/>
+      <c r="I266" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
@@ -10488,7 +10558,9 @@
       </c>
       <c r="G267" s="1" t="inlineStr"/>
       <c r="H267" s="1" t="inlineStr"/>
-      <c r="I267" s="1" t="inlineStr"/>
+      <c r="I267" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
@@ -10521,7 +10593,9 @@
       </c>
       <c r="G268" s="1" t="inlineStr"/>
       <c r="H268" s="1" t="inlineStr"/>
-      <c r="I268" s="1" t="inlineStr"/>
+      <c r="I268" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
@@ -10554,7 +10628,9 @@
       </c>
       <c r="G269" s="1" t="inlineStr"/>
       <c r="H269" s="1" t="inlineStr"/>
-      <c r="I269" s="1" t="inlineStr"/>
+      <c r="I269" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
@@ -10587,7 +10663,9 @@
       </c>
       <c r="G270" s="1" t="inlineStr"/>
       <c r="H270" s="1" t="inlineStr"/>
-      <c r="I270" s="1" t="inlineStr"/>
+      <c r="I270" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
@@ -10620,7 +10698,9 @@
       </c>
       <c r="G271" s="1" t="inlineStr"/>
       <c r="H271" s="1" t="inlineStr"/>
-      <c r="I271" s="1" t="inlineStr"/>
+      <c r="I271" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
@@ -11657,7 +11737,9 @@
       <c r="F298" s="2" t="inlineStr"/>
       <c r="G298" s="1" t="inlineStr"/>
       <c r="H298" s="1" t="inlineStr"/>
-      <c r="I298" s="1" t="inlineStr"/>
+      <c r="I298" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
@@ -11688,7 +11770,9 @@
       </c>
       <c r="G299" s="1" t="inlineStr"/>
       <c r="H299" s="1" t="inlineStr"/>
-      <c r="I299" s="1" t="inlineStr"/>
+      <c r="I299" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
@@ -11719,7 +11803,9 @@
       </c>
       <c r="G300" s="1" t="inlineStr"/>
       <c r="H300" s="1" t="inlineStr"/>
-      <c r="I300" s="1" t="inlineStr"/>
+      <c r="I300" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
@@ -13031,7 +13117,9 @@
       <c r="F334" s="2" t="inlineStr"/>
       <c r="G334" s="1" t="inlineStr"/>
       <c r="H334" s="1" t="inlineStr"/>
-      <c r="I334" s="1" t="inlineStr"/>
+      <c r="I334" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
@@ -13064,7 +13152,9 @@
       </c>
       <c r="G335" s="1" t="inlineStr"/>
       <c r="H335" s="1" t="inlineStr"/>
-      <c r="I335" s="1" t="inlineStr"/>
+      <c r="I335" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
@@ -13097,7 +13187,9 @@
       </c>
       <c r="G336" s="1" t="inlineStr"/>
       <c r="H336" s="1" t="inlineStr"/>
-      <c r="I336" s="1" t="inlineStr"/>
+      <c r="I336" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
@@ -13130,7 +13222,9 @@
       </c>
       <c r="G337" s="1" t="inlineStr"/>
       <c r="H337" s="1" t="inlineStr"/>
-      <c r="I337" s="1" t="inlineStr"/>
+      <c r="I337" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
@@ -13163,7 +13257,9 @@
       </c>
       <c r="G338" s="1" t="inlineStr"/>
       <c r="H338" s="1" t="inlineStr"/>
-      <c r="I338" s="1" t="inlineStr"/>
+      <c r="I338" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
@@ -14157,7 +14253,9 @@
       <c r="F364" s="2" t="inlineStr"/>
       <c r="G364" s="1" t="inlineStr"/>
       <c r="H364" s="1" t="inlineStr"/>
-      <c r="I364" s="1" t="inlineStr"/>
+      <c r="I364" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
@@ -14190,7 +14288,9 @@
       </c>
       <c r="G365" s="1" t="inlineStr"/>
       <c r="H365" s="1" t="inlineStr"/>
-      <c r="I365" s="1" t="inlineStr"/>
+      <c r="I365" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
@@ -14221,7 +14321,9 @@
       </c>
       <c r="G366" s="1" t="inlineStr"/>
       <c r="H366" s="1" t="inlineStr"/>
-      <c r="I366" s="1" t="inlineStr"/>
+      <c r="I366" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
@@ -14252,7 +14354,9 @@
       </c>
       <c r="G367" s="1" t="inlineStr"/>
       <c r="H367" s="1" t="inlineStr"/>
-      <c r="I367" s="1" t="inlineStr"/>
+      <c r="I367" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
@@ -14283,7 +14387,9 @@
       </c>
       <c r="G368" s="1" t="inlineStr"/>
       <c r="H368" s="1" t="inlineStr"/>
-      <c r="I368" s="1" t="inlineStr"/>
+      <c r="I368" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
@@ -15004,7 +15110,9 @@
       <c r="F387" s="2" t="inlineStr"/>
       <c r="G387" s="1" t="inlineStr"/>
       <c r="H387" s="1" t="inlineStr"/>
-      <c r="I387" s="1" t="inlineStr"/>
+      <c r="I387" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="1" t="inlineStr">
@@ -15037,7 +15145,9 @@
       </c>
       <c r="G388" s="1" t="inlineStr"/>
       <c r="H388" s="1" t="inlineStr"/>
-      <c r="I388" s="1" t="inlineStr"/>
+      <c r="I388" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="389">
       <c r="A389" s="1" t="inlineStr">
@@ -15068,7 +15178,9 @@
       </c>
       <c r="G389" s="1" t="inlineStr"/>
       <c r="H389" s="1" t="inlineStr"/>
-      <c r="I389" s="1" t="inlineStr"/>
+      <c r="I389" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="390">
       <c r="A390" s="1" t="inlineStr">
@@ -15099,7 +15211,9 @@
       </c>
       <c r="G390" s="1" t="inlineStr"/>
       <c r="H390" s="1" t="inlineStr"/>
-      <c r="I390" s="1" t="inlineStr"/>
+      <c r="I390" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="391">
       <c r="A391" s="1" t="inlineStr">
@@ -15132,7 +15246,9 @@
       </c>
       <c r="G391" s="1" t="inlineStr"/>
       <c r="H391" s="1" t="inlineStr"/>
-      <c r="I391" s="1" t="inlineStr"/>
+      <c r="I391" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="1" t="inlineStr">
@@ -15165,7 +15281,9 @@
       </c>
       <c r="G392" s="1" t="inlineStr"/>
       <c r="H392" s="1" t="inlineStr"/>
-      <c r="I392" s="1" t="inlineStr"/>
+      <c r="I392" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="393">
       <c r="A393" s="1" t="inlineStr">
@@ -15198,7 +15316,9 @@
       </c>
       <c r="G393" s="1" t="inlineStr"/>
       <c r="H393" s="1" t="inlineStr"/>
-      <c r="I393" s="1" t="inlineStr"/>
+      <c r="I393" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="394">
       <c r="A394" s="1" t="inlineStr">
@@ -15960,7 +16080,9 @@
       <c r="F413" s="2" t="inlineStr"/>
       <c r="G413" s="1" t="inlineStr"/>
       <c r="H413" s="1" t="inlineStr"/>
-      <c r="I413" s="1" t="inlineStr"/>
+      <c r="I413" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="414">
       <c r="A414" s="1" t="inlineStr">
@@ -15991,7 +16113,9 @@
       </c>
       <c r="G414" s="1" t="inlineStr"/>
       <c r="H414" s="1" t="inlineStr"/>
-      <c r="I414" s="1" t="inlineStr"/>
+      <c r="I414" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="415">
       <c r="A415" s="1" t="inlineStr">
@@ -16024,7 +16148,9 @@
       </c>
       <c r="G415" s="1" t="inlineStr"/>
       <c r="H415" s="1" t="inlineStr"/>
-      <c r="I415" s="1" t="inlineStr"/>
+      <c r="I415" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="416">
       <c r="A416" s="1" t="inlineStr">
@@ -16663,7 +16789,9 @@
       <c r="F432" s="2" t="inlineStr"/>
       <c r="G432" s="1" t="inlineStr"/>
       <c r="H432" s="1" t="inlineStr"/>
-      <c r="I432" s="1" t="inlineStr"/>
+      <c r="I432" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="433">
       <c r="A433" s="1" t="inlineStr">
@@ -16694,7 +16822,9 @@
       </c>
       <c r="G433" s="1" t="inlineStr"/>
       <c r="H433" s="1" t="inlineStr"/>
-      <c r="I433" s="1" t="inlineStr"/>
+      <c r="I433" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="434">
       <c r="A434" s="1" t="inlineStr">
@@ -16727,7 +16857,9 @@
       </c>
       <c r="G434" s="1" t="inlineStr"/>
       <c r="H434" s="1" t="inlineStr"/>
-      <c r="I434" s="1" t="inlineStr"/>
+      <c r="I434" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="435">
       <c r="A435" s="1" t="inlineStr">
@@ -16760,7 +16892,9 @@
       </c>
       <c r="G435" s="1" t="inlineStr"/>
       <c r="H435" s="1" t="inlineStr"/>
-      <c r="I435" s="1" t="inlineStr"/>
+      <c r="I435" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="436">
       <c r="A436" s="1" t="inlineStr">
@@ -16793,7 +16927,9 @@
       </c>
       <c r="G436" s="1" t="inlineStr"/>
       <c r="H436" s="1" t="inlineStr"/>
-      <c r="I436" s="1" t="inlineStr"/>
+      <c r="I436" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="437">
       <c r="A437" s="1" t="inlineStr">
@@ -17596,7 +17732,9 @@
       <c r="F457" s="2" t="inlineStr"/>
       <c r="G457" s="1" t="inlineStr"/>
       <c r="H457" s="1" t="inlineStr"/>
-      <c r="I457" s="1" t="inlineStr"/>
+      <c r="I457" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="458">
       <c r="A458" s="1" t="inlineStr">
@@ -17629,7 +17767,9 @@
       </c>
       <c r="G458" s="1" t="inlineStr"/>
       <c r="H458" s="1" t="inlineStr"/>
-      <c r="I458" s="1" t="inlineStr"/>
+      <c r="I458" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="459">
       <c r="A459" s="1" t="inlineStr">
@@ -17662,7 +17802,9 @@
       </c>
       <c r="G459" s="1" t="inlineStr"/>
       <c r="H459" s="1" t="inlineStr"/>
-      <c r="I459" s="1" t="inlineStr"/>
+      <c r="I459" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="460">
       <c r="A460" s="1" t="inlineStr">
@@ -17695,7 +17837,9 @@
       </c>
       <c r="G460" s="1" t="inlineStr"/>
       <c r="H460" s="1" t="inlineStr"/>
-      <c r="I460" s="1" t="inlineStr"/>
+      <c r="I460" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="461">
       <c r="A461" s="1" t="inlineStr">
@@ -19151,7 +19295,9 @@
       <c r="F498" s="2" t="inlineStr"/>
       <c r="G498" s="1" t="inlineStr"/>
       <c r="H498" s="1" t="inlineStr"/>
-      <c r="I498" s="1" t="inlineStr"/>
+      <c r="I498" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="499">
       <c r="A499" s="1" t="inlineStr">
@@ -19184,7 +19330,9 @@
       </c>
       <c r="G499" s="1" t="inlineStr"/>
       <c r="H499" s="1" t="inlineStr"/>
-      <c r="I499" s="1" t="inlineStr"/>
+      <c r="I499" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="500">
       <c r="A500" s="1" t="inlineStr">
@@ -19217,7 +19365,9 @@
       </c>
       <c r="G500" s="1" t="inlineStr"/>
       <c r="H500" s="1" t="inlineStr"/>
-      <c r="I500" s="1" t="inlineStr"/>
+      <c r="I500" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="501">
       <c r="A501" s="1" t="inlineStr">
@@ -19250,7 +19400,9 @@
       </c>
       <c r="G501" s="1" t="inlineStr"/>
       <c r="H501" s="1" t="inlineStr"/>
-      <c r="I501" s="1" t="inlineStr"/>
+      <c r="I501" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="502">
       <c r="A502" s="1" t="inlineStr">
@@ -19283,7 +19435,9 @@
       </c>
       <c r="G502" s="1" t="inlineStr"/>
       <c r="H502" s="1" t="inlineStr"/>
-      <c r="I502" s="1" t="inlineStr"/>
+      <c r="I502" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="503">
       <c r="A503" s="1" t="inlineStr">
@@ -19316,7 +19470,9 @@
       </c>
       <c r="G503" s="1" t="inlineStr"/>
       <c r="H503" s="1" t="inlineStr"/>
-      <c r="I503" s="1" t="inlineStr"/>
+      <c r="I503" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="504">
       <c r="A504" s="1" t="inlineStr">
@@ -20312,7 +20468,9 @@
       <c r="F529" s="2" t="inlineStr"/>
       <c r="G529" s="1" t="inlineStr"/>
       <c r="H529" s="1" t="inlineStr"/>
-      <c r="I529" s="1" t="inlineStr"/>
+      <c r="I529" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="530">
       <c r="A530" s="1" t="inlineStr">
@@ -20345,7 +20503,9 @@
       </c>
       <c r="G530" s="1" t="inlineStr"/>
       <c r="H530" s="1" t="inlineStr"/>
-      <c r="I530" s="1" t="inlineStr"/>
+      <c r="I530" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="531">
       <c r="A531" s="1" t="inlineStr">
@@ -20376,7 +20536,9 @@
       </c>
       <c r="G531" s="1" t="inlineStr"/>
       <c r="H531" s="1" t="inlineStr"/>
-      <c r="I531" s="1" t="inlineStr"/>
+      <c r="I531" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="532">
       <c r="A532" s="1" t="inlineStr">
@@ -21688,7 +21850,9 @@
       <c r="F565" s="2" t="inlineStr"/>
       <c r="G565" s="1" t="inlineStr"/>
       <c r="H565" s="1" t="inlineStr"/>
-      <c r="I565" s="1" t="inlineStr"/>
+      <c r="I565" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="566">
       <c r="A566" s="1" t="inlineStr">
@@ -21721,7 +21885,9 @@
       </c>
       <c r="G566" s="1" t="inlineStr"/>
       <c r="H566" s="1" t="inlineStr"/>
-      <c r="I566" s="1" t="inlineStr"/>
+      <c r="I566" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="567">
       <c r="A567" s="1" t="inlineStr">
@@ -21754,7 +21920,9 @@
       </c>
       <c r="G567" s="1" t="inlineStr"/>
       <c r="H567" s="1" t="inlineStr"/>
-      <c r="I567" s="1" t="inlineStr"/>
+      <c r="I567" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="568">
       <c r="A568" s="1" t="inlineStr">
@@ -21787,7 +21955,9 @@
       </c>
       <c r="G568" s="1" t="inlineStr"/>
       <c r="H568" s="1" t="inlineStr"/>
-      <c r="I568" s="1" t="inlineStr"/>
+      <c r="I568" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="569">
       <c r="A569" s="1" t="inlineStr">
@@ -21820,7 +21990,9 @@
       </c>
       <c r="G569" s="1" t="inlineStr"/>
       <c r="H569" s="1" t="inlineStr"/>
-      <c r="I569" s="1" t="inlineStr"/>
+      <c r="I569" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="570">
       <c r="A570" s="1" t="inlineStr">
@@ -22816,7 +22988,9 @@
       <c r="F595" s="2" t="inlineStr"/>
       <c r="G595" s="1" t="inlineStr"/>
       <c r="H595" s="1" t="inlineStr"/>
-      <c r="I595" s="1" t="inlineStr"/>
+      <c r="I595" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="596">
       <c r="A596" s="1" t="inlineStr">
@@ -22849,7 +23023,9 @@
       </c>
       <c r="G596" s="1" t="inlineStr"/>
       <c r="H596" s="1" t="inlineStr"/>
-      <c r="I596" s="1" t="inlineStr"/>
+      <c r="I596" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="597">
       <c r="A597" s="1" t="inlineStr">
@@ -22882,7 +23058,9 @@
       </c>
       <c r="G597" s="1" t="inlineStr"/>
       <c r="H597" s="1" t="inlineStr"/>
-      <c r="I597" s="1" t="inlineStr"/>
+      <c r="I597" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="598">
       <c r="A598" s="1" t="inlineStr">
@@ -22915,7 +23093,9 @@
       </c>
       <c r="G598" s="1" t="inlineStr"/>
       <c r="H598" s="1" t="inlineStr"/>
-      <c r="I598" s="1" t="inlineStr"/>
+      <c r="I598" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="599">
       <c r="A599" s="1" t="inlineStr">
@@ -22948,7 +23128,9 @@
       </c>
       <c r="G599" s="1" t="inlineStr"/>
       <c r="H599" s="1" t="inlineStr"/>
-      <c r="I599" s="1" t="inlineStr"/>
+      <c r="I599" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="600">
       <c r="A600" s="1" t="inlineStr">
@@ -23669,7 +23851,9 @@
       <c r="F618" s="2" t="inlineStr"/>
       <c r="G618" s="1" t="inlineStr"/>
       <c r="H618" s="1" t="inlineStr"/>
-      <c r="I618" s="1" t="inlineStr"/>
+      <c r="I618" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="619">
       <c r="A619" s="1" t="inlineStr">
@@ -23702,7 +23886,9 @@
       </c>
       <c r="G619" s="1" t="inlineStr"/>
       <c r="H619" s="1" t="inlineStr"/>
-      <c r="I619" s="1" t="inlineStr"/>
+      <c r="I619" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="620">
       <c r="A620" s="1" t="inlineStr">
@@ -23733,7 +23919,9 @@
       </c>
       <c r="G620" s="1" t="inlineStr"/>
       <c r="H620" s="1" t="inlineStr"/>
-      <c r="I620" s="1" t="inlineStr"/>
+      <c r="I620" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="621">
       <c r="A621" s="1" t="inlineStr">
@@ -23764,7 +23952,9 @@
       </c>
       <c r="G621" s="1" t="inlineStr"/>
       <c r="H621" s="1" t="inlineStr"/>
-      <c r="I621" s="1" t="inlineStr"/>
+      <c r="I621" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="622">
       <c r="A622" s="1" t="inlineStr">
@@ -23797,7 +23987,9 @@
       </c>
       <c r="G622" s="1" t="inlineStr"/>
       <c r="H622" s="1" t="inlineStr"/>
-      <c r="I622" s="1" t="inlineStr"/>
+      <c r="I622" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="623">
       <c r="A623" s="1" t="inlineStr">
@@ -23830,7 +24022,9 @@
       </c>
       <c r="G623" s="1" t="inlineStr"/>
       <c r="H623" s="1" t="inlineStr"/>
-      <c r="I623" s="1" t="inlineStr"/>
+      <c r="I623" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="624">
       <c r="A624" s="1" t="inlineStr">
@@ -23863,7 +24057,9 @@
       </c>
       <c r="G624" s="1" t="inlineStr"/>
       <c r="H624" s="1" t="inlineStr"/>
-      <c r="I624" s="1" t="inlineStr"/>
+      <c r="I624" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="625">
       <c r="A625" s="1" t="inlineStr">
@@ -24625,7 +24821,9 @@
       <c r="F644" s="2" t="inlineStr"/>
       <c r="G644" s="1" t="inlineStr"/>
       <c r="H644" s="1" t="inlineStr"/>
-      <c r="I644" s="1" t="inlineStr"/>
+      <c r="I644" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="645">
       <c r="A645" s="1" t="inlineStr">
@@ -24656,7 +24854,9 @@
       </c>
       <c r="G645" s="1" t="inlineStr"/>
       <c r="H645" s="1" t="inlineStr"/>
-      <c r="I645" s="1" t="inlineStr"/>
+      <c r="I645" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="646">
       <c r="A646" s="1" t="inlineStr">
@@ -24689,7 +24889,9 @@
       </c>
       <c r="G646" s="1" t="inlineStr"/>
       <c r="H646" s="1" t="inlineStr"/>
-      <c r="I646" s="1" t="inlineStr"/>
+      <c r="I646" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="647">
       <c r="A647" s="1" t="inlineStr">
@@ -25328,7 +25530,9 @@
       <c r="F663" s="2" t="inlineStr"/>
       <c r="G663" s="1" t="inlineStr"/>
       <c r="H663" s="1" t="inlineStr"/>
-      <c r="I663" s="1" t="inlineStr"/>
+      <c r="I663" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="664">
       <c r="A664" s="1" t="inlineStr">
@@ -25359,7 +25563,9 @@
       </c>
       <c r="G664" s="1" t="inlineStr"/>
       <c r="H664" s="1" t="inlineStr"/>
-      <c r="I664" s="1" t="inlineStr"/>
+      <c r="I664" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="665">
       <c r="A665" s="1" t="inlineStr">
@@ -25392,7 +25598,9 @@
       </c>
       <c r="G665" s="1" t="inlineStr"/>
       <c r="H665" s="1" t="inlineStr"/>
-      <c r="I665" s="1" t="inlineStr"/>
+      <c r="I665" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="666">
       <c r="A666" s="1" t="inlineStr">
@@ -25425,7 +25633,9 @@
       </c>
       <c r="G666" s="1" t="inlineStr"/>
       <c r="H666" s="1" t="inlineStr"/>
-      <c r="I666" s="1" t="inlineStr"/>
+      <c r="I666" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="667">
       <c r="A667" s="1" t="inlineStr">
@@ -25458,7 +25668,9 @@
       </c>
       <c r="G667" s="1" t="inlineStr"/>
       <c r="H667" s="1" t="inlineStr"/>
-      <c r="I667" s="1" t="inlineStr"/>
+      <c r="I667" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="668">
       <c r="A668" s="1" t="inlineStr">
@@ -26261,7 +26473,9 @@
       <c r="F688" s="2" t="inlineStr"/>
       <c r="G688" s="1" t="inlineStr"/>
       <c r="H688" s="1" t="inlineStr"/>
-      <c r="I688" s="1" t="inlineStr"/>
+      <c r="I688" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="689">
       <c r="A689" s="1" t="inlineStr">
@@ -26294,7 +26508,9 @@
       </c>
       <c r="G689" s="1" t="inlineStr"/>
       <c r="H689" s="1" t="inlineStr"/>
-      <c r="I689" s="1" t="inlineStr"/>
+      <c r="I689" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="690">
       <c r="A690" s="1" t="inlineStr">
@@ -26327,7 +26543,9 @@
       </c>
       <c r="G690" s="1" t="inlineStr"/>
       <c r="H690" s="1" t="inlineStr"/>
-      <c r="I690" s="1" t="inlineStr"/>
+      <c r="I690" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="691">
       <c r="A691" s="1" t="inlineStr">
@@ -26360,7 +26578,9 @@
       </c>
       <c r="G691" s="1" t="inlineStr"/>
       <c r="H691" s="1" t="inlineStr"/>
-      <c r="I691" s="1" t="inlineStr"/>
+      <c r="I691" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="692">
       <c r="A692" s="1" t="inlineStr">
@@ -26393,7 +26613,9 @@
       </c>
       <c r="G692" s="1" t="inlineStr"/>
       <c r="H692" s="1" t="inlineStr"/>
-      <c r="I692" s="1" t="inlineStr"/>
+      <c r="I692" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="693">
       <c r="A693" s="1" t="inlineStr">
@@ -27847,7 +28069,9 @@
       <c r="F730" s="2" t="inlineStr"/>
       <c r="G730" s="1" t="inlineStr"/>
       <c r="H730" s="1" t="inlineStr"/>
-      <c r="I730" s="1" t="inlineStr"/>
+      <c r="I730" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="731">
       <c r="A731" s="1" t="inlineStr">
@@ -27880,7 +28104,9 @@
       </c>
       <c r="G731" s="1" t="inlineStr"/>
       <c r="H731" s="1" t="inlineStr"/>
-      <c r="I731" s="1" t="inlineStr"/>
+      <c r="I731" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="732">
       <c r="A732" s="1" t="inlineStr">
@@ -27913,7 +28139,9 @@
       </c>
       <c r="G732" s="1" t="inlineStr"/>
       <c r="H732" s="1" t="inlineStr"/>
-      <c r="I732" s="1" t="inlineStr"/>
+      <c r="I732" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="733">
       <c r="A733" s="1" t="inlineStr">
@@ -27946,7 +28174,9 @@
       </c>
       <c r="G733" s="1" t="inlineStr"/>
       <c r="H733" s="1" t="inlineStr"/>
-      <c r="I733" s="1" t="inlineStr"/>
+      <c r="I733" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="734">
       <c r="A734" s="1" t="inlineStr">
@@ -27979,7 +28209,9 @@
       </c>
       <c r="G734" s="1" t="inlineStr"/>
       <c r="H734" s="1" t="inlineStr"/>
-      <c r="I734" s="1" t="inlineStr"/>
+      <c r="I734" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="735">
       <c r="A735" s="1" t="inlineStr">
@@ -28973,7 +29205,9 @@
       <c r="F760" s="2" t="inlineStr"/>
       <c r="G760" s="1" t="inlineStr"/>
       <c r="H760" s="1" t="inlineStr"/>
-      <c r="I760" s="1" t="inlineStr"/>
+      <c r="I760" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="761">
       <c r="A761" s="1" t="inlineStr">
@@ -29004,7 +29238,9 @@
       </c>
       <c r="G761" s="1" t="inlineStr"/>
       <c r="H761" s="1" t="inlineStr"/>
-      <c r="I761" s="1" t="inlineStr"/>
+      <c r="I761" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="762">
       <c r="A762" s="1" t="inlineStr">
@@ -29035,7 +29271,9 @@
       </c>
       <c r="G762" s="1" t="inlineStr"/>
       <c r="H762" s="1" t="inlineStr"/>
-      <c r="I762" s="1" t="inlineStr"/>
+      <c r="I762" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="763">
       <c r="A763" s="1" t="inlineStr">
@@ -29066,7 +29304,9 @@
       </c>
       <c r="G763" s="1" t="inlineStr"/>
       <c r="H763" s="1" t="inlineStr"/>
-      <c r="I763" s="1" t="inlineStr"/>
+      <c r="I763" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="764">
       <c r="A764" s="1" t="inlineStr">
@@ -30378,7 +30618,9 @@
       <c r="F797" s="2" t="inlineStr"/>
       <c r="G797" s="1" t="inlineStr"/>
       <c r="H797" s="1" t="inlineStr"/>
-      <c r="I797" s="1" t="inlineStr"/>
+      <c r="I797" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="798">
       <c r="A798" s="1" t="inlineStr">
@@ -30411,7 +30653,9 @@
       </c>
       <c r="G798" s="1" t="inlineStr"/>
       <c r="H798" s="1" t="inlineStr"/>
-      <c r="I798" s="1" t="inlineStr"/>
+      <c r="I798" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="799">
       <c r="A799" s="1" t="inlineStr">
@@ -30444,7 +30688,9 @@
       </c>
       <c r="G799" s="1" t="inlineStr"/>
       <c r="H799" s="1" t="inlineStr"/>
-      <c r="I799" s="1" t="inlineStr"/>
+      <c r="I799" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="800">
       <c r="A800" s="1" t="inlineStr">
@@ -30477,7 +30723,9 @@
       </c>
       <c r="G800" s="1" t="inlineStr"/>
       <c r="H800" s="1" t="inlineStr"/>
-      <c r="I800" s="1" t="inlineStr"/>
+      <c r="I800" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="801">
       <c r="A801" s="1" t="inlineStr">
@@ -31473,7 +31721,9 @@
       <c r="F826" s="2" t="inlineStr"/>
       <c r="G826" s="1" t="inlineStr"/>
       <c r="H826" s="1" t="inlineStr"/>
-      <c r="I826" s="1" t="inlineStr"/>
+      <c r="I826" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="827">
       <c r="A827" s="1" t="inlineStr">
@@ -31506,7 +31756,9 @@
       </c>
       <c r="G827" s="1" t="inlineStr"/>
       <c r="H827" s="1" t="inlineStr"/>
-      <c r="I827" s="1" t="inlineStr"/>
+      <c r="I827" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="828">
       <c r="A828" s="1" t="inlineStr">
@@ -31539,7 +31791,9 @@
       </c>
       <c r="G828" s="1" t="inlineStr"/>
       <c r="H828" s="1" t="inlineStr"/>
-      <c r="I828" s="1" t="inlineStr"/>
+      <c r="I828" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="829">
       <c r="A829" s="1" t="inlineStr">
@@ -32260,7 +32514,9 @@
       <c r="F847" s="2" t="inlineStr"/>
       <c r="G847" s="1" t="inlineStr"/>
       <c r="H847" s="1" t="inlineStr"/>
-      <c r="I847" s="1" t="inlineStr"/>
+      <c r="I847" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="848">
       <c r="A848" s="1" t="inlineStr">
@@ -32293,7 +32549,9 @@
       </c>
       <c r="G848" s="1" t="inlineStr"/>
       <c r="H848" s="1" t="inlineStr"/>
-      <c r="I848" s="1" t="inlineStr"/>
+      <c r="I848" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="849">
       <c r="A849" s="1" t="inlineStr">
@@ -32326,7 +32584,9 @@
       </c>
       <c r="G849" s="1" t="inlineStr"/>
       <c r="H849" s="1" t="inlineStr"/>
-      <c r="I849" s="1" t="inlineStr"/>
+      <c r="I849" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="850">
       <c r="A850" s="1" t="inlineStr">
@@ -33088,7 +33348,9 @@
       <c r="F869" s="2" t="inlineStr"/>
       <c r="G869" s="1" t="inlineStr"/>
       <c r="H869" s="1" t="inlineStr"/>
-      <c r="I869" s="1" t="inlineStr"/>
+      <c r="I869" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="870">
       <c r="A870" s="1" t="inlineStr">
@@ -33121,7 +33383,9 @@
       </c>
       <c r="G870" s="1" t="inlineStr"/>
       <c r="H870" s="1" t="inlineStr"/>
-      <c r="I870" s="1" t="inlineStr"/>
+      <c r="I870" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="871">
       <c r="A871" s="1" t="inlineStr">
@@ -33760,7 +34024,9 @@
       <c r="F887" s="2" t="inlineStr"/>
       <c r="G887" s="1" t="inlineStr"/>
       <c r="H887" s="1" t="inlineStr"/>
-      <c r="I887" s="1" t="inlineStr"/>
+      <c r="I887" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="888">
       <c r="A888" s="1" t="inlineStr">
@@ -33793,7 +34059,9 @@
       </c>
       <c r="G888" s="1" t="inlineStr"/>
       <c r="H888" s="1" t="inlineStr"/>
-      <c r="I888" s="1" t="inlineStr"/>
+      <c r="I888" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="889">
       <c r="A889" s="1" t="inlineStr">
@@ -33826,7 +34094,9 @@
       </c>
       <c r="G889" s="1" t="inlineStr"/>
       <c r="H889" s="1" t="inlineStr"/>
-      <c r="I889" s="1" t="inlineStr"/>
+      <c r="I889" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="890">
       <c r="A890" s="1" t="inlineStr">
@@ -33859,7 +34129,9 @@
       </c>
       <c r="G890" s="1" t="inlineStr"/>
       <c r="H890" s="1" t="inlineStr"/>
-      <c r="I890" s="1" t="inlineStr"/>
+      <c r="I890" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="891">
       <c r="A891" s="1" t="inlineStr">
@@ -34662,7 +34934,9 @@
       <c r="F911" s="2" t="inlineStr"/>
       <c r="G911" s="1" t="inlineStr"/>
       <c r="H911" s="1" t="inlineStr"/>
-      <c r="I911" s="1" t="inlineStr"/>
+      <c r="I911" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="912">
       <c r="A912" s="1" t="inlineStr">
@@ -34695,7 +34969,9 @@
       </c>
       <c r="G912" s="1" t="inlineStr"/>
       <c r="H912" s="1" t="inlineStr"/>
-      <c r="I912" s="1" t="inlineStr"/>
+      <c r="I912" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="913">
       <c r="A913" s="1" t="inlineStr">
@@ -34728,7 +35004,9 @@
       </c>
       <c r="G913" s="1" t="inlineStr"/>
       <c r="H913" s="1" t="inlineStr"/>
-      <c r="I913" s="1" t="inlineStr"/>
+      <c r="I913" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="914">
       <c r="A914" s="1" t="inlineStr">
@@ -36184,7 +36462,9 @@
       <c r="F951" s="2" t="inlineStr"/>
       <c r="G951" s="1" t="inlineStr"/>
       <c r="H951" s="1" t="inlineStr"/>
-      <c r="I951" s="1" t="inlineStr"/>
+      <c r="I951" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="952">
       <c r="A952" s="1" t="inlineStr">
@@ -36217,7 +36497,9 @@
       </c>
       <c r="G952" s="1" t="inlineStr"/>
       <c r="H952" s="1" t="inlineStr"/>
-      <c r="I952" s="1" t="inlineStr"/>
+      <c r="I952" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="953">
       <c r="A953" s="1" t="inlineStr">
@@ -36250,7 +36532,9 @@
       </c>
       <c r="G953" s="1" t="inlineStr"/>
       <c r="H953" s="1" t="inlineStr"/>
-      <c r="I953" s="1" t="inlineStr"/>
+      <c r="I953" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="954">
       <c r="A954" s="1" t="inlineStr">
@@ -36283,7 +36567,9 @@
       </c>
       <c r="G954" s="1" t="inlineStr"/>
       <c r="H954" s="1" t="inlineStr"/>
-      <c r="I954" s="1" t="inlineStr"/>
+      <c r="I954" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="955">
       <c r="A955" s="1" t="inlineStr">
@@ -37279,7 +37565,9 @@
       <c r="F980" s="2" t="inlineStr"/>
       <c r="G980" s="1" t="inlineStr"/>
       <c r="H980" s="1" t="inlineStr"/>
-      <c r="I980" s="1" t="inlineStr"/>
+      <c r="I980" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="981">
       <c r="A981" s="1" t="inlineStr">
@@ -37312,7 +37600,9 @@
       </c>
       <c r="G981" s="1" t="inlineStr"/>
       <c r="H981" s="1" t="inlineStr"/>
-      <c r="I981" s="1" t="inlineStr"/>
+      <c r="I981" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="982">
       <c r="A982" s="1" t="inlineStr">
@@ -37345,7 +37635,9 @@
       </c>
       <c r="G982" s="1" t="inlineStr"/>
       <c r="H982" s="1" t="inlineStr"/>
-      <c r="I982" s="1" t="inlineStr"/>
+      <c r="I982" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="983">
       <c r="A983" s="1" t="inlineStr">
@@ -37378,7 +37670,9 @@
       </c>
       <c r="G983" s="1" t="inlineStr"/>
       <c r="H983" s="1" t="inlineStr"/>
-      <c r="I983" s="1" t="inlineStr"/>
+      <c r="I983" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="984">
       <c r="A984" s="1" t="inlineStr">
@@ -38690,7 +38984,9 @@
       <c r="F1017" s="2" t="inlineStr"/>
       <c r="G1017" s="1" t="inlineStr"/>
       <c r="H1017" s="1" t="inlineStr"/>
-      <c r="I1017" s="1" t="inlineStr"/>
+      <c r="I1017" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1018">
       <c r="A1018" s="1" t="inlineStr">
@@ -38723,7 +39019,9 @@
       </c>
       <c r="G1018" s="1" t="inlineStr"/>
       <c r="H1018" s="1" t="inlineStr"/>
-      <c r="I1018" s="1" t="inlineStr"/>
+      <c r="I1018" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1019">
       <c r="A1019" s="1" t="inlineStr">
@@ -38756,7 +39054,9 @@
       </c>
       <c r="G1019" s="1" t="inlineStr"/>
       <c r="H1019" s="1" t="inlineStr"/>
-      <c r="I1019" s="1" t="inlineStr"/>
+      <c r="I1019" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1020">
       <c r="A1020" s="1" t="inlineStr">
@@ -38789,7 +39089,9 @@
       </c>
       <c r="G1020" s="1" t="inlineStr"/>
       <c r="H1020" s="1" t="inlineStr"/>
-      <c r="I1020" s="1" t="inlineStr"/>
+      <c r="I1020" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1021">
       <c r="A1021" s="1" t="inlineStr">
@@ -39785,7 +40087,9 @@
       <c r="F1046" s="2" t="inlineStr"/>
       <c r="G1046" s="1" t="inlineStr"/>
       <c r="H1046" s="1" t="inlineStr"/>
-      <c r="I1046" s="1" t="inlineStr"/>
+      <c r="I1046" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1047">
       <c r="A1047" s="1" t="inlineStr">
@@ -39818,7 +40122,9 @@
       </c>
       <c r="G1047" s="1" t="inlineStr"/>
       <c r="H1047" s="1" t="inlineStr"/>
-      <c r="I1047" s="1" t="inlineStr"/>
+      <c r="I1047" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1048">
       <c r="A1048" s="1" t="inlineStr">
@@ -39851,7 +40157,9 @@
       </c>
       <c r="G1048" s="1" t="inlineStr"/>
       <c r="H1048" s="1" t="inlineStr"/>
-      <c r="I1048" s="1" t="inlineStr"/>
+      <c r="I1048" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1049">
       <c r="A1049" s="1" t="inlineStr">
@@ -40572,7 +40880,9 @@
       <c r="F1067" s="2" t="inlineStr"/>
       <c r="G1067" s="1" t="inlineStr"/>
       <c r="H1067" s="1" t="inlineStr"/>
-      <c r="I1067" s="1" t="inlineStr"/>
+      <c r="I1067" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1068">
       <c r="A1068" s="1" t="inlineStr">
@@ -40605,7 +40915,9 @@
       </c>
       <c r="G1068" s="1" t="inlineStr"/>
       <c r="H1068" s="1" t="inlineStr"/>
-      <c r="I1068" s="1" t="inlineStr"/>
+      <c r="I1068" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1069">
       <c r="A1069" s="1" t="inlineStr">
@@ -40638,7 +40950,9 @@
       </c>
       <c r="G1069" s="1" t="inlineStr"/>
       <c r="H1069" s="1" t="inlineStr"/>
-      <c r="I1069" s="1" t="inlineStr"/>
+      <c r="I1069" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1070">
       <c r="A1070" s="1" t="inlineStr">
@@ -40671,7 +40985,9 @@
       </c>
       <c r="G1070" s="1" t="inlineStr"/>
       <c r="H1070" s="1" t="inlineStr"/>
-      <c r="I1070" s="1" t="inlineStr"/>
+      <c r="I1070" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1071">
       <c r="A1071" s="1" t="inlineStr">
@@ -40704,7 +41020,9 @@
       </c>
       <c r="G1071" s="1" t="inlineStr"/>
       <c r="H1071" s="1" t="inlineStr"/>
-      <c r="I1071" s="1" t="inlineStr"/>
+      <c r="I1071" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1072">
       <c r="A1072" s="1" t="inlineStr">
@@ -41466,7 +41784,9 @@
       <c r="F1091" s="2" t="inlineStr"/>
       <c r="G1091" s="1" t="inlineStr"/>
       <c r="H1091" s="1" t="inlineStr"/>
-      <c r="I1091" s="1" t="inlineStr"/>
+      <c r="I1091" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1092">
       <c r="A1092" s="1" t="inlineStr">
@@ -41499,7 +41819,9 @@
       </c>
       <c r="G1092" s="1" t="inlineStr"/>
       <c r="H1092" s="1" t="inlineStr"/>
-      <c r="I1092" s="1" t="inlineStr"/>
+      <c r="I1092" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1093">
       <c r="A1093" s="1" t="inlineStr">
@@ -42138,7 +42460,9 @@
       <c r="F1109" s="2" t="inlineStr"/>
       <c r="G1109" s="1" t="inlineStr"/>
       <c r="H1109" s="1" t="inlineStr"/>
-      <c r="I1109" s="1" t="inlineStr"/>
+      <c r="I1109" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1110">
       <c r="A1110" s="1" t="inlineStr">
@@ -42171,7 +42495,9 @@
       </c>
       <c r="G1110" s="1" t="inlineStr"/>
       <c r="H1110" s="1" t="inlineStr"/>
-      <c r="I1110" s="1" t="inlineStr"/>
+      <c r="I1110" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1111">
       <c r="A1111" s="1" t="inlineStr">
@@ -42204,7 +42530,9 @@
       </c>
       <c r="G1111" s="1" t="inlineStr"/>
       <c r="H1111" s="1" t="inlineStr"/>
-      <c r="I1111" s="1" t="inlineStr"/>
+      <c r="I1111" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1112">
       <c r="A1112" s="1" t="inlineStr">
@@ -42237,7 +42565,9 @@
       </c>
       <c r="G1112" s="1" t="inlineStr"/>
       <c r="H1112" s="1" t="inlineStr"/>
-      <c r="I1112" s="1" t="inlineStr"/>
+      <c r="I1112" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1113">
       <c r="A1113" s="1" t="inlineStr">
@@ -43040,7 +43370,9 @@
       <c r="F1133" s="2" t="inlineStr"/>
       <c r="G1133" s="1" t="inlineStr"/>
       <c r="H1133" s="1" t="inlineStr"/>
-      <c r="I1133" s="1" t="inlineStr"/>
+      <c r="I1133" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1134">
       <c r="A1134" s="1" t="inlineStr">
@@ -43073,7 +43405,9 @@
       </c>
       <c r="G1134" s="1" t="inlineStr"/>
       <c r="H1134" s="1" t="inlineStr"/>
-      <c r="I1134" s="1" t="inlineStr"/>
+      <c r="I1134" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1135">
       <c r="A1135" s="1" t="inlineStr">
@@ -43106,7 +43440,9 @@
       </c>
       <c r="G1135" s="1" t="inlineStr"/>
       <c r="H1135" s="1" t="inlineStr"/>
-      <c r="I1135" s="1" t="inlineStr"/>
+      <c r="I1135" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1136">
       <c r="A1136" s="1" t="inlineStr">
@@ -43139,7 +43475,9 @@
       </c>
       <c r="G1136" s="1" t="inlineStr"/>
       <c r="H1136" s="1" t="inlineStr"/>
-      <c r="I1136" s="1" t="inlineStr"/>
+      <c r="I1136" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1137">
       <c r="A1137" s="1" t="inlineStr">
@@ -43172,7 +43510,9 @@
       </c>
       <c r="G1137" s="1" t="inlineStr"/>
       <c r="H1137" s="1" t="inlineStr"/>
-      <c r="I1137" s="1" t="inlineStr"/>
+      <c r="I1137" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1138">
       <c r="A1138" s="1" t="inlineStr">

</xml_diff>